<commit_message>
Show steps to fix as numbered steps
- App: Steps to fix is now a numbered list, one box per step; Enter adds
  the next step, Backspace joins steps, pasting several lines makes
  several steps, plus an Add step button
- Excel guide and app download: step numbers in bold

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Np6FjV33ZtJzjSs2EYKhw9
</commit_message>
<xml_diff>
--- a/Error Code Guide - UNI-300VA Labeler.xlsx
+++ b/Error Code Guide - UNI-300VA Labeler.xlsx
@@ -614,12 +614,113 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>1. Stop the line and pull the rejected bottles
-2. Look at the rejects: label straight? code clear and correct?
-3. Check the label roll is the right item # for this batch
-4. Fix what you found (see the matching error below)
-5. Reset the error and restart the line
-6. Watch the next bottles and tell your lead</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line and pull the rejected bottles</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Look at the rejects: label straight? code clear and correct?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the label roll is the right item # for this batch</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Fix what you found (see the matching error below)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+5. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+6. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Watch the next bottles and tell your lead</t>
+          </r>
         </is>
       </c>
     </row>
@@ -656,11 +757,95 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>1. Pull the affected bottles and set them aside for QA
-2. Check the code on the label matches the batch record
-3. Check the coder ribbon (see ribbon errors)
-4. Reset the error and restart the line
-5. Tell your lead / QA</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Pull the affected bottles and set them aside for QA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the code on the label matches the batch record</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the coder ribbon (see ribbon errors)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+5. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Tell your lead / QA</t>
+          </r>
         </is>
       </c>
     </row>
@@ -697,10 +882,77 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1. Pull the unlabeled bottles
-2. Check the label roll and that the web follows the threading diagram
-3. Remove any stuck or folded labels
-4. Reset the error and restart the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Pull the unlabeled bottles</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the label roll and that the web follows the threading diagram</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Remove any stuck or folded labels</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
         </is>
       </c>
     </row>
@@ -735,10 +987,77 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>1. Get the next roll ready
-2. Check the item # and lot match the batch record
-3. Change the roll when it runs out
-4. Record the roll change</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Get the next roll ready</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the item # and lot match the batch record</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Change the roll when it runs out</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Record the roll change</t>
+          </r>
         </is>
       </c>
     </row>
@@ -773,12 +1092,113 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>1. Stop the line
-2. Load the new roll (check item # and lot)
-3. Thread the web using the diagram on the machine
-4. Record the roll change
-5. Reset the error and restart the line
-6. Check the first labeled bottles</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Load the new roll (check item # and lot)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Thread the web using the diagram on the machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Record the roll change</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+5. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+6. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the first labeled bottles</t>
+          </r>
         </is>
       </c>
     </row>
@@ -815,11 +1235,95 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>1. Stop the line
-2. Remove the torn liner
-3. Re-thread the web using the diagram on the machine
-4. Reset the error and restart the line
-5. Check the first labeled bottles</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Remove the torn liner</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Re-thread the web using the diagram on the machine</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+5. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the first labeled bottles</t>
+          </r>
         </is>
       </c>
     </row>
@@ -854,12 +1358,113 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>1. Stop the line
-2. Open the coder cassette and replace the ribbon
-3. Follow the threading diagram inside the cassette
-4. Close and lock the cassette
-5. Check the screen shows RUNNING
-6. Restart the line and check the first codes</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Open the coder cassette and replace the ribbon</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Follow the threading diagram inside the cassette</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Close and lock the cassette</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+5. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the screen shows RUNNING</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+6. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Restart the line and check the first codes</t>
+          </r>
         </is>
       </c>
     </row>
@@ -896,11 +1501,95 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>1. Stop the line
-2. Open the cassette and re-thread or replace the ribbon
-3. Close and lock the cassette
-4. Clear the message on the coder screen
-5. Restart the line and check the first codes</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Open the cassette and re-thread or replace the ribbon</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Close and lock the cassette</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Clear the message on the coder screen</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+5. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Restart the line and check the first codes</t>
+          </r>
         </is>
       </c>
     </row>
@@ -937,10 +1626,77 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>1. Check the message on the Videojet screen and clear it
-2. Make sure the correct job is selected and matches the batch record
-3. Press start - the screen should show green RUNNING
-4. Restart the line and check the first codes</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Check the message on the Videojet screen and clear it</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Make sure the correct job is selected and matches the batch record</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Press start - the screen should show green RUNNING</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+4. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Restart the line and check the first codes</t>
+          </r>
         </is>
       </c>
     </row>
@@ -976,9 +1732,59 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>1. Stop the line before reaching in
-2. Remove the fallen or jammed bottles
-3. Reset the error and restart the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line before reaching in</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Remove the fallen or jammed bottles</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
         </is>
       </c>
     </row>
@@ -1014,9 +1820,59 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>1. Stop the line
-2. Remove the stuck bottle at the indexing wheel
-3. Reset the error and restart the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Stop the line</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Remove the stuck bottle at the indexing wheel</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
         </is>
       </c>
     </row>
@@ -1051,8 +1907,41 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>1. Empty the reject bin and keep rejects separate
-2. Reset the error and restart the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Empty the reject bin and keep rejects separate</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
         </is>
       </c>
     </row>
@@ -1087,8 +1976,41 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>1. Close all guard doors until they latch
-2. Reset the error and restart the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Close all guard doors until they latch</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
         </is>
       </c>
     </row>
@@ -1123,9 +2045,59 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>1. Make sure the area is safe and everyone is clear
-2. Twist or pull the E-stop button to release it
-3. Reset the error and restart the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">1. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Make sure the area is safe and everyone is clear</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+2. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Twist or pull the E-stop button to release it</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+3. </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reset the error and restart the line</t>
+          </r>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show possible problems as bullet points
- App: Possible problem uses the same list editor as the steps, with
  bullets: Enter for the next problem, Backspace to join, paste lines,
  Add problem button
- Excel guide and app download: bold bullets
- Column dividers span the full row; guides dropdown fits on phones

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Np6FjV33ZtJzjSs2EYKhw9
</commit_message>
<xml_diff>
--- a/Error Code Guide - UNI-300VA Labeler.xlsx
+++ b/Error Code Guide - UNI-300VA Labeler.xlsx
@@ -607,9 +607,59 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>• Labels crooked or wrinkled
-• Lot / exp code missing, faded or wrong
-• Wrong label roll loaded</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Labels crooked or wrinkled</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Lot / exp code missing, faded or wrong</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Wrong label roll loaded</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -750,9 +800,59 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>• Lot / exp code missing or faded
-• Ribbon wrinkled or running out
-• Wrong code loaded on the coder</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Lot / exp code missing or faded</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Ribbon wrinkled or running out</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Wrong code loaded on the coder</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
@@ -875,9 +975,59 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>• Labeler ran out of labels
-• Labels stuck to each other or to the liner
-• Label web not threaded right</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Labeler ran out of labels</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Labels stuck to each other or to the liner</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Label web not threaded right</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -982,7 +1132,23 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>• Label roll is almost empty</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Label roll is almost empty</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -1087,7 +1253,23 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>• Label roll is empty</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Label roll is empty</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1228,9 +1410,59 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>• Label liner torn
-• Liner caught on a guide
-• Bad splice in the roll</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Label liner torn</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Liner caught on a guide</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Bad splice in the roll</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -1353,7 +1585,23 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>• Coder ribbon almost used up or empty</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Coder ribbon almost used up or empty</t>
+          </r>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1494,9 +1742,59 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>• Ribbon torn or slipped off
-• Ribbon threaded wrong
-• Cassette not locked</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Ribbon torn or slipped off</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Ribbon threaded wrong</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Cassette not locked</t>
+          </r>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -1619,9 +1917,59 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>• Coder is stopped or paused
-• Cassette open or message not cleared
-• No job (code) selected</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Coder is stopped or paused</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Cassette open or message not cleared</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>No job (code) selected</t>
+          </r>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1726,8 +2074,41 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>• Bottle fell over or got stuck
-• Damaged or wrong bottles on the line</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Bottle fell over or got stuck</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Damaged or wrong bottles on the line</t>
+          </r>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -1814,8 +2195,41 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>• Bottle stuck at the indexing wheel
-• Bottles crowded at the infeed</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Bottle stuck at the indexing wheel</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">
+• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Bottles crowded at the infeed</t>
+          </r>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1902,7 +2316,23 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>• Reject bin is full</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Reject bin is full</t>
+          </r>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -1971,7 +2401,23 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>• A guard door is open or not fully closed</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>A guard door is open or not fully closed</t>
+          </r>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -2040,7 +2486,23 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>• Someone pressed the red E-stop button</t>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <b val="1"/>
+              <color rgb="001F3A4D"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">• </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Aptos Narrow"/>
+              <color rgb="00222222"/>
+              <sz val="13"/>
+            </rPr>
+            <t>Someone pressed the red E-stop button</t>
+          </r>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">

</xml_diff>